<commit_message>
Implemented process identification, dashboard logging and alerts
</commit_message>
<xml_diff>
--- a/mlmodel/training_data.xlsx
+++ b/mlmodel/training_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1012"/>
+  <dimension ref="A1:G1038"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23718,6 +23718,604 @@
         <v>0.705</v>
       </c>
     </row>
+    <row r="1013">
+      <c r="A1013" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1013" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1013" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1013" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1013" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1013" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1013" t="n">
+        <v>0.777</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1014" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1014" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1014" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1014" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1014" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1014" t="n">
+        <v>0.476</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1015" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1015" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1015" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1015" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1015" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1015" t="n">
+        <v>0.476</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1016" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1016" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1016" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1016" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1016" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1016" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1017" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1017" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1017" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1017" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1017" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1017" t="n">
+        <v>0.46</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1018" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1018" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1018" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1018" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1018" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1018" t="n">
+        <v>0.5620000000000001</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1019" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1019" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1019" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1019" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1019" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1019" t="n">
+        <v>0.5620000000000001</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1020" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1020" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1020" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1020" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1020" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1020" t="n">
+        <v>0.589</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1021" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1021" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1021" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1021" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1021" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1021" t="n">
+        <v>0.589</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1022" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1022" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1022" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1022" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1022" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1022" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1023" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1023" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1023" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1023" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1023" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1023" t="n">
+        <v>0.58</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1024" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1024" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1024" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1024" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1024" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1024" t="n">
+        <v>0.8159999999999999</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1025" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1025" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1025" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1025" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1025" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1025" t="n">
+        <v>0.443</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1026" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1026" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1026" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1026" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1026" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1026" t="n">
+        <v>0.421</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1027" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1027" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1027" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1027" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1027" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1027" t="n">
+        <v>0.648</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1028" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1028" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1028" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1028" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1028" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1028" t="n">
+        <v>0.477</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1029" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1029" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1029" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1029" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1029" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1029" t="n">
+        <v>0.233</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1030" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1030" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1030" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1030" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1030" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1030" t="n">
+        <v>0.577</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1031" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1031" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1031" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1031" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1031" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1031" t="n">
+        <v>0.698</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1032" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1032" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1032" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1032" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1032" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1032" t="n">
+        <v>0.294</v>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1033" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1033" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1033" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1033" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1033" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1033" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1034" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1034" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1034" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1034" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1034" t="n">
+        <v>1</v>
+      </c>
+      <c r="G1034" t="n">
+        <v>2.331</v>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1035" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1035" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1035" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1035" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1035" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1035" t="n">
+        <v>0.21</v>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1036" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1036" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1036" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1036" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1036" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1036" t="n">
+        <v>0.308</v>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1037" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1037" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1037" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1037" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1037" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1037" t="n">
+        <v>0.419</v>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1038" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1038" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1038" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1038" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1038" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1038" t="n">
+        <v>0.495</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Implemented alerts page and fixed alerts API to filter suspicious webcam activity
</commit_message>
<xml_diff>
--- a/mlmodel/training_data.xlsx
+++ b/mlmodel/training_data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1038"/>
+  <dimension ref="A1:G1046"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24316,6 +24316,190 @@
         <v>0.495</v>
       </c>
     </row>
+    <row r="1039">
+      <c r="A1039" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1039" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1039" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1039" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1039" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1039" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1039" t="n">
+        <v>0.378</v>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1040" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1040" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1040" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1040" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1040" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1040" t="n">
+        <v>0.402</v>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1041" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1041" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1041" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1041" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1041" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1041" t="n">
+        <v>0.384</v>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1042" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1042" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1042" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1042" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1042" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1042" t="n">
+        <v>0.346</v>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1043" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1043" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1043" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1043" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1043" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1043" t="n">
+        <v>0.312</v>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1044" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1044" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1044" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1044" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1044" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1044" t="n">
+        <v>0.346</v>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1045" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1045" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1045" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1045" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1045" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1045" t="n">
+        <v>0.426</v>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1046" t="n">
+        <v>0</v>
+      </c>
+      <c r="C1046" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1046" t="n">
+        <v>1</v>
+      </c>
+      <c r="E1046" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1046" t="n">
+        <v>2</v>
+      </c>
+      <c r="G1046" t="n">
+        <v>0.387</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>